<commit_message>
Precharge notifications: add Technical Section Leader to the rig-side recipients
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HKpkuLyV6bHMBgkcjiDHio
</commit_message>
<xml_diff>
--- a/WCE_Precharge_Notification.xlsx
+++ b/WCE_Precharge_Notification.xlsx
@@ -153,13 +153,14 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Rigs" displayName="Rigs" ref="A1:D14" headerRowCount="1">
-  <autoFilter ref="A1:D14"/>
-  <tableColumns count="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Rigs" displayName="Rigs" ref="A1:E14" headerRowCount="1">
+  <autoFilter ref="A1:E14"/>
+  <tableColumns count="5">
     <tableColumn id="1" name="Vessel"/>
     <tableColumn id="2" name="RigKey"/>
     <tableColumn id="3" name="SubseaSupervisorName"/>
     <tableColumn id="4" name="SubseaSupervisorEmail"/>
+    <tableColumn id="5" name="TSLEmail"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
@@ -480,7 +481,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Rigs     - one row per rig: the rig's Subsea Supervisor. Fill the yellow cells. Vessel must match meta.asset in the files exactly; RigKey is the calculator's short code (already filled) and is used when a request carries no rig name.</t>
+          <t>Rigs     - one row per rig: the rig's Subsea Supervisor and Technical Section Leader (TSLEmail). Fill the yellow cells. Vessel must match meta.asset in the files exactly; RigKey is the calculator's short code (already filled) and is used when a request carries no rig name.</t>
         </is>
       </c>
     </row>
@@ -504,7 +505,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Issued precharge posted from the calculator (seadrill-report_..._precharge.json)  -&gt;  TO that rig's Subsea Supervisor, CC the Office table.</t>
+          <t xml:space="preserve">  Issued precharge posted from the calculator (seadrill-report_..._precharge.json)  -&gt;  TO that rig's Subsea Supervisor and TSL, CC the Office table.</t>
         </is>
       </c>
     </row>
@@ -602,13 +603,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -632,6 +634,11 @@
           <t>SubseaSupervisorEmail</t>
         </is>
       </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>TSLEmail</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -646,6 +653,7 @@
       </c>
       <c r="C2" s="3" t="inlineStr"/>
       <c r="D2" s="3" t="inlineStr"/>
+      <c r="E2" s="3" t="n"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -660,6 +668,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr"/>
       <c r="D3" s="3" t="inlineStr"/>
+      <c r="E3" s="3" t="n"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -674,6 +683,11 @@
       </c>
       <c r="C4" s="3" t="inlineStr"/>
       <c r="D4" s="3" t="inlineStr"/>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>TSL.wVela@seadrill.com</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -688,6 +702,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr"/>
       <c r="D5" s="3" t="inlineStr"/>
+      <c r="E5" s="3" t="n"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -702,6 +717,7 @@
       </c>
       <c r="C6" s="3" t="inlineStr"/>
       <c r="D6" s="3" t="inlineStr"/>
+      <c r="E6" s="3" t="n"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -716,6 +732,7 @@
       </c>
       <c r="C7" s="3" t="inlineStr"/>
       <c r="D7" s="3" t="inlineStr"/>
+      <c r="E7" s="3" t="n"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -730,6 +747,7 @@
       </c>
       <c r="C8" s="3" t="inlineStr"/>
       <c r="D8" s="3" t="inlineStr"/>
+      <c r="E8" s="3" t="n"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -744,6 +762,7 @@
       </c>
       <c r="C9" s="3" t="inlineStr"/>
       <c r="D9" s="3" t="inlineStr"/>
+      <c r="E9" s="3" t="n"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -758,6 +777,7 @@
       </c>
       <c r="C10" s="3" t="inlineStr"/>
       <c r="D10" s="3" t="inlineStr"/>
+      <c r="E10" s="3" t="n"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -772,6 +792,7 @@
       </c>
       <c r="C11" s="3" t="inlineStr"/>
       <c r="D11" s="3" t="inlineStr"/>
+      <c r="E11" s="3" t="n"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -786,6 +807,7 @@
       </c>
       <c r="C12" s="3" t="inlineStr"/>
       <c r="D12" s="3" t="inlineStr"/>
+      <c r="E12" s="3" t="n"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -800,6 +822,7 @@
       </c>
       <c r="C13" s="3" t="inlineStr"/>
       <c r="D13" s="3" t="inlineStr"/>
+      <c r="E13" s="3" t="n"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -814,6 +837,7 @@
       </c>
       <c r="C14" s="3" t="inlineStr"/>
       <c r="D14" s="3" t="inlineStr"/>
+      <c r="E14" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>